<commit_message>
Product: quick start guide, debt order fix, richer sample data
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product/Tidy-Money-Budget-Dashboard.xlsx
+++ b/product/Tidy-Money-Budget-Dashboard.xlsx
@@ -1473,7 +1473,7 @@
         <v>3200</v>
       </c>
       <c r="J7" s="42" t="n">
-        <v>21300</v>
+        <v>8900</v>
       </c>
       <c r="K7" s="42" t="n">
         <v>0</v>
@@ -1519,7 +1519,7 @@
         <v>3050</v>
       </c>
       <c r="J8" s="42" t="n">
-        <v>21035</v>
+        <v>8635</v>
       </c>
       <c r="K8" s="42" t="n">
         <v>0</v>
@@ -1568,7 +1568,7 @@
         <v>2900</v>
       </c>
       <c r="J9" s="42" t="n">
-        <v>20770</v>
+        <v>8370</v>
       </c>
       <c r="K9" s="42" t="n">
         <v>0</v>
@@ -5590,169 +5590,481 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="35" t="n"/>
-      <c r="C23" s="32" t="n"/>
-      <c r="D23" s="32" t="n"/>
-      <c r="E23" s="32" t="n"/>
-      <c r="F23" s="36" t="n"/>
-      <c r="G23" s="32" t="n"/>
-      <c r="H23" s="32" t="n"/>
+      <c r="B23" s="35" t="n">
+        <v>46267</v>
+      </c>
+      <c r="C23" s="32" t="inlineStr">
+        <is>
+          <t>Doctor copay</t>
+        </is>
+      </c>
+      <c r="D23" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E23" s="32" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="F23" s="36" t="n">
+        <v>40</v>
+      </c>
+      <c r="G23" s="32" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="H23" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I23" s="37">
         <f>IF(B23="","",DATE(YEAR(B23),MONTH(B23),1))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="35" t="n"/>
-      <c r="C24" s="32" t="n"/>
-      <c r="D24" s="32" t="n"/>
-      <c r="E24" s="32" t="n"/>
-      <c r="F24" s="36" t="n"/>
-      <c r="G24" s="32" t="n"/>
-      <c r="H24" s="32" t="n"/>
+      <c r="B24" s="35" t="n">
+        <v>46270</v>
+      </c>
+      <c r="C24" s="32" t="inlineStr">
+        <is>
+          <t>Grocery run</t>
+        </is>
+      </c>
+      <c r="D24" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E24" s="32" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="F24" s="36" t="n">
+        <v>115.2</v>
+      </c>
+      <c r="G24" s="32" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="H24" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I24" s="37">
         <f>IF(B24="","",DATE(YEAR(B24),MONTH(B24),1))</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="35" t="n"/>
-      <c r="C25" s="32" t="n"/>
-      <c r="D25" s="32" t="n"/>
-      <c r="E25" s="32" t="n"/>
-      <c r="F25" s="36" t="n"/>
-      <c r="G25" s="32" t="n"/>
-      <c r="H25" s="32" t="n"/>
+      <c r="B25" s="35" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C25" s="32" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="D25" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E25" s="32" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="F25" s="36" t="n">
+        <v>48</v>
+      </c>
+      <c r="G25" s="32" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="H25" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I25" s="37">
         <f>IF(B25="","",DATE(YEAR(B25),MONTH(B25),1))</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="35" t="n"/>
-      <c r="C26" s="32" t="n"/>
-      <c r="D26" s="32" t="n"/>
-      <c r="E26" s="32" t="n"/>
-      <c r="F26" s="36" t="n"/>
-      <c r="G26" s="32" t="n"/>
-      <c r="H26" s="32" t="n"/>
+      <c r="B26" s="35" t="n">
+        <v>46276</v>
+      </c>
+      <c r="C26" s="32" t="inlineStr">
+        <is>
+          <t>Music app</t>
+        </is>
+      </c>
+      <c r="D26" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E26" s="32" t="inlineStr">
+        <is>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="F26" s="36" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="G26" s="32" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="H26" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I26" s="37">
         <f>IF(B26="","",DATE(YEAR(B26),MONTH(B26),1))</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="35" t="n"/>
-      <c r="C27" s="32" t="n"/>
-      <c r="D27" s="32" t="n"/>
-      <c r="E27" s="32" t="n"/>
-      <c r="F27" s="36" t="n"/>
-      <c r="G27" s="32" t="n"/>
-      <c r="H27" s="32" t="n"/>
+      <c r="B27" s="35" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C27" s="32" t="inlineStr">
+        <is>
+          <t>Haircut</t>
+        </is>
+      </c>
+      <c r="D27" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E27" s="32" t="inlineStr">
+        <is>
+          <t>Personal care</t>
+        </is>
+      </c>
+      <c r="F27" s="36" t="n">
+        <v>35</v>
+      </c>
+      <c r="G27" s="32" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="H27" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I27" s="37">
         <f>IF(B27="","",DATE(YEAR(B27),MONTH(B27),1))</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="35" t="n"/>
-      <c r="C28" s="32" t="n"/>
-      <c r="D28" s="32" t="n"/>
-      <c r="E28" s="32" t="n"/>
-      <c r="F28" s="36" t="n"/>
-      <c r="G28" s="32" t="n"/>
-      <c r="H28" s="32" t="n"/>
+      <c r="B28" s="35" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C28" s="32" t="inlineStr">
+        <is>
+          <t>Grocery run</t>
+        </is>
+      </c>
+      <c r="D28" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E28" s="32" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="F28" s="36" t="n">
+        <v>131.6</v>
+      </c>
+      <c r="G28" s="32" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="H28" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I28" s="37">
         <f>IF(B28="","",DATE(YEAR(B28),MONTH(B28),1))</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="35" t="n"/>
-      <c r="C29" s="32" t="n"/>
-      <c r="D29" s="32" t="n"/>
-      <c r="E29" s="32" t="n"/>
-      <c r="F29" s="36" t="n"/>
-      <c r="G29" s="32" t="n"/>
-      <c r="H29" s="32" t="n"/>
+      <c r="B29" s="35" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C29" s="32" t="inlineStr">
+        <is>
+          <t>Water bill</t>
+        </is>
+      </c>
+      <c r="D29" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E29" s="32" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="F29" s="36" t="n">
+        <v>45</v>
+      </c>
+      <c r="G29" s="32" t="inlineStr">
+        <is>
+          <t>Checking</t>
+        </is>
+      </c>
+      <c r="H29" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I29" s="37">
         <f>IF(B29="","",DATE(YEAR(B29),MONTH(B29),1))</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="35" t="n"/>
-      <c r="C30" s="32" t="n"/>
-      <c r="D30" s="32" t="n"/>
-      <c r="E30" s="32" t="n"/>
-      <c r="F30" s="36" t="n"/>
-      <c r="G30" s="32" t="n"/>
-      <c r="H30" s="32" t="n"/>
+      <c r="B30" s="35" t="n">
+        <v>46288</v>
+      </c>
+      <c r="C30" s="32" t="inlineStr">
+        <is>
+          <t>Birthday gift</t>
+        </is>
+      </c>
+      <c r="D30" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E30" s="32" t="inlineStr">
+        <is>
+          <t>Gifts &amp; giving</t>
+        </is>
+      </c>
+      <c r="F30" s="36" t="n">
+        <v>40</v>
+      </c>
+      <c r="G30" s="32" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="H30" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I30" s="37">
         <f>IF(B30="","",DATE(YEAR(B30),MONTH(B30),1))</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="35" t="n"/>
-      <c r="C31" s="32" t="n"/>
-      <c r="D31" s="32" t="n"/>
-      <c r="E31" s="32" t="n"/>
-      <c r="F31" s="36" t="n"/>
-      <c r="G31" s="32" t="n"/>
-      <c r="H31" s="32" t="n"/>
+      <c r="B31" s="35" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C31" s="32" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="D31" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E31" s="32" t="inlineStr">
+        <is>
+          <t>Eating out</t>
+        </is>
+      </c>
+      <c r="F31" s="36" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="G31" s="32" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="H31" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I31" s="37">
         <f>IF(B31="","",DATE(YEAR(B31),MONTH(B31),1))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="35" t="n"/>
-      <c r="C32" s="32" t="n"/>
-      <c r="D32" s="32" t="n"/>
-      <c r="E32" s="32" t="n"/>
-      <c r="F32" s="36" t="n"/>
-      <c r="G32" s="32" t="n"/>
-      <c r="H32" s="32" t="n"/>
+      <c r="B32" s="35" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C32" s="32" t="inlineStr">
+        <is>
+          <t>Grocery run</t>
+        </is>
+      </c>
+      <c r="D32" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E32" s="32" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="F32" s="36" t="n">
+        <v>120.35</v>
+      </c>
+      <c r="G32" s="32" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="H32" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I32" s="37">
         <f>IF(B32="","",DATE(YEAR(B32),MONTH(B32),1))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="35" t="n"/>
-      <c r="C33" s="32" t="n"/>
-      <c r="D33" s="32" t="n"/>
-      <c r="E33" s="32" t="n"/>
-      <c r="F33" s="36" t="n"/>
-      <c r="G33" s="32" t="n"/>
-      <c r="H33" s="32" t="n"/>
+      <c r="B33" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C33" s="32" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D33" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E33" s="32" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="F33" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="G33" s="32" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="H33" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I33" s="37">
         <f>IF(B33="","",DATE(YEAR(B33),MONTH(B33),1))</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="35" t="n"/>
-      <c r="C34" s="32" t="n"/>
-      <c r="D34" s="32" t="n"/>
-      <c r="E34" s="32" t="n"/>
-      <c r="F34" s="36" t="n"/>
-      <c r="G34" s="32" t="n"/>
-      <c r="H34" s="32" t="n"/>
+      <c r="B34" s="35" t="n">
+        <v>46294</v>
+      </c>
+      <c r="C34" s="32" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="D34" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E34" s="32" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="F34" s="36" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="G34" s="32" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="H34" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I34" s="37">
         <f>IF(B34="","",DATE(YEAR(B34),MONTH(B34),1))</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="35" t="n"/>
-      <c r="C35" s="32" t="n"/>
-      <c r="D35" s="32" t="n"/>
-      <c r="E35" s="32" t="n"/>
-      <c r="F35" s="36" t="n"/>
-      <c r="G35" s="32" t="n"/>
-      <c r="H35" s="32" t="n"/>
+      <c r="B35" s="35" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C35" s="32" t="inlineStr">
+        <is>
+          <t>Credit card payment</t>
+        </is>
+      </c>
+      <c r="D35" s="32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E35" s="32" t="inlineStr">
+        <is>
+          <t>Debt payments</t>
+        </is>
+      </c>
+      <c r="F35" s="36" t="n">
+        <v>250</v>
+      </c>
+      <c r="G35" s="32" t="inlineStr">
+        <is>
+          <t>Checking</t>
+        </is>
+      </c>
+      <c r="H35" s="32" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
       <c r="I35" s="37">
         <f>IF(B35="","",DATE(YEAR(B35),MONTH(B35),1))</f>
         <v/>
@@ -24699,7 +25011,7 @@
         <v>95</v>
       </c>
       <c r="F8" s="46">
-        <f>IF(B8="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C8,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C8,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C8,C8,$B$8:$B8,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D8,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D8,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D8,D8,$B$8:$B8,"&lt;&gt;")+1))</f>
+        <f>IF(B8="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C8))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C8)*(ROW($B$8:$B$22)&lt;8))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D8))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D8)*(ROW($B$8:$B$22)&lt;8))+1))</f>
         <v/>
       </c>
       <c r="G8" s="46">
@@ -24732,7 +25044,7 @@
         <v>265</v>
       </c>
       <c r="F9" s="46">
-        <f>IF(B9="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C9,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C9,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C9,C9,$B$8:$B9,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D9,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D9,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D9,D9,$B$8:$B9,"&lt;&gt;")+1))</f>
+        <f>IF(B9="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C9))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C9)*(ROW($B$8:$B$22)&lt;9))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D9))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D9)*(ROW($B$8:$B$22)&lt;9))+1))</f>
         <v/>
       </c>
       <c r="G9" s="46">
@@ -24765,7 +25077,7 @@
         <v>140</v>
       </c>
       <c r="F10" s="46">
-        <f>IF(B10="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C10,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C10,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C10,C10,$B$8:$B10,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D10,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D10,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D10,D10,$B$8:$B10,"&lt;&gt;")+1))</f>
+        <f>IF(B10="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C10))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C10)*(ROW($B$8:$B$22)&lt;10))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D10))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D10)*(ROW($B$8:$B$22)&lt;10))+1))</f>
         <v/>
       </c>
       <c r="G10" s="46">
@@ -24798,7 +25110,7 @@
         <v>30</v>
       </c>
       <c r="F11" s="46">
-        <f>IF(B11="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C11,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C11,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C11,C11,$B$8:$B11,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D11,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D11,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D11,D11,$B$8:$B11,"&lt;&gt;")+1))</f>
+        <f>IF(B11="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C11))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C11)*(ROW($B$8:$B$22)&lt;11))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D11))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D11)*(ROW($B$8:$B$22)&lt;11))+1))</f>
         <v/>
       </c>
       <c r="G11" s="46">
@@ -24821,7 +25133,7 @@
       <c r="D12" s="51" t="n"/>
       <c r="E12" s="42" t="n"/>
       <c r="F12" s="46">
-        <f>IF(B12="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C12,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C12,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C12,C12,$B$8:$B12,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D12,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D12,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D12,D12,$B$8:$B12,"&lt;&gt;")+1))</f>
+        <f>IF(B12="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C12))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C12)*(ROW($B$8:$B$22)&lt;12))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D12))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D12)*(ROW($B$8:$B$22)&lt;12))+1))</f>
         <v/>
       </c>
       <c r="G12" s="46">
@@ -24844,7 +25156,7 @@
       <c r="D13" s="51" t="n"/>
       <c r="E13" s="42" t="n"/>
       <c r="F13" s="46">
-        <f>IF(B13="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C13,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C13,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C13,C13,$B$8:$B13,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D13,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D13,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D13,D13,$B$8:$B13,"&lt;&gt;")+1))</f>
+        <f>IF(B13="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C13))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C13)*(ROW($B$8:$B$22)&lt;13))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D13))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D13)*(ROW($B$8:$B$22)&lt;13))+1))</f>
         <v/>
       </c>
       <c r="G13" s="46">
@@ -24867,7 +25179,7 @@
       <c r="D14" s="51" t="n"/>
       <c r="E14" s="42" t="n"/>
       <c r="F14" s="46">
-        <f>IF(B14="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C14,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C14,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C14,C14,$B$8:$B14,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D14,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D14,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D14,D14,$B$8:$B14,"&lt;&gt;")+1))</f>
+        <f>IF(B14="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C14))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C14)*(ROW($B$8:$B$22)&lt;14))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D14))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D14)*(ROW($B$8:$B$22)&lt;14))+1))</f>
         <v/>
       </c>
       <c r="G14" s="46">
@@ -24890,7 +25202,7 @@
       <c r="D15" s="51" t="n"/>
       <c r="E15" s="42" t="n"/>
       <c r="F15" s="46">
-        <f>IF(B15="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C15,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C15,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C15,C15,$B$8:$B15,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D15,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D15,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D15,D15,$B$8:$B15,"&lt;&gt;")+1))</f>
+        <f>IF(B15="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C15))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C15)*(ROW($B$8:$B$22)&lt;15))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D15))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D15)*(ROW($B$8:$B$22)&lt;15))+1))</f>
         <v/>
       </c>
       <c r="G15" s="46">
@@ -24913,7 +25225,7 @@
       <c r="D16" s="51" t="n"/>
       <c r="E16" s="42" t="n"/>
       <c r="F16" s="46">
-        <f>IF(B16="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C16,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C16,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C16,C16,$B$8:$B16,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D16,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D16,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D16,D16,$B$8:$B16,"&lt;&gt;")+1))</f>
+        <f>IF(B16="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C16))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C16)*(ROW($B$8:$B$22)&lt;16))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D16))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D16)*(ROW($B$8:$B$22)&lt;16))+1))</f>
         <v/>
       </c>
       <c r="G16" s="46">
@@ -24936,7 +25248,7 @@
       <c r="D17" s="51" t="n"/>
       <c r="E17" s="42" t="n"/>
       <c r="F17" s="46">
-        <f>IF(B17="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C17,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C17,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C17,C17,$B$8:$B17,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D17,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D17,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D17,D17,$B$8:$B17,"&lt;&gt;")+1))</f>
+        <f>IF(B17="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C17))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C17)*(ROW($B$8:$B$22)&lt;17))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D17))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D17)*(ROW($B$8:$B$22)&lt;17))+1))</f>
         <v/>
       </c>
       <c r="G17" s="46">
@@ -24959,7 +25271,7 @@
       <c r="D18" s="51" t="n"/>
       <c r="E18" s="42" t="n"/>
       <c r="F18" s="46">
-        <f>IF(B18="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C18,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C18,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C18,C18,$B$8:$B18,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D18,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D18,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D18,D18,$B$8:$B18,"&lt;&gt;")+1))</f>
+        <f>IF(B18="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C18))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C18)*(ROW($B$8:$B$22)&lt;18))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D18))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D18)*(ROW($B$8:$B$22)&lt;18))+1))</f>
         <v/>
       </c>
       <c r="G18" s="46">
@@ -24982,7 +25294,7 @@
       <c r="D19" s="51" t="n"/>
       <c r="E19" s="42" t="n"/>
       <c r="F19" s="46">
-        <f>IF(B19="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C19,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C19,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C19,C19,$B$8:$B19,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D19,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D19,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D19,D19,$B$8:$B19,"&lt;&gt;")+1))</f>
+        <f>IF(B19="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C19))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C19)*(ROW($B$8:$B$22)&lt;19))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D19))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D19)*(ROW($B$8:$B$22)&lt;19))+1))</f>
         <v/>
       </c>
       <c r="G19" s="46">
@@ -25005,7 +25317,7 @@
       <c r="D20" s="51" t="n"/>
       <c r="E20" s="42" t="n"/>
       <c r="F20" s="46">
-        <f>IF(B20="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C20,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C20,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C20,C20,$B$8:$B20,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D20,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D20,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D20,D20,$B$8:$B20,"&lt;&gt;")+1))</f>
+        <f>IF(B20="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C20))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C20)*(ROW($B$8:$B$22)&lt;20))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D20))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D20)*(ROW($B$8:$B$22)&lt;20))+1))</f>
         <v/>
       </c>
       <c r="G20" s="46">
@@ -25028,7 +25340,7 @@
       <c r="D21" s="51" t="n"/>
       <c r="E21" s="42" t="n"/>
       <c r="F21" s="46">
-        <f>IF(B21="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C21,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C21,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C21,C21,$B$8:$B21,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D21,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D21,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D21,D21,$B$8:$B21,"&lt;&gt;")+1))</f>
+        <f>IF(B21="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C21))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C21)*(ROW($B$8:$B$22)&lt;21))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D21))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D21)*(ROW($B$8:$B$22)&lt;21))+1))</f>
         <v/>
       </c>
       <c r="G21" s="46">
@@ -25051,7 +25363,7 @@
       <c r="D22" s="51" t="n"/>
       <c r="E22" s="42" t="n"/>
       <c r="F22" s="46">
-        <f>IF(B22="","",IF($C$5="Snowball",COUNTIFS($C$8:$C$22,"&lt;"&amp;C22,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($C$8:$C$22,C22,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($C$8:$C22,C22,$B$8:$B22,"&lt;&gt;")+1,COUNTIFS($D$8:$D$22,"&gt;"&amp;D22,$B$8:$B$22,"&lt;&gt;")+COUNTIFS($D$8:$D$22,D22,$B$8:$B$22,"&lt;&gt;")-COUNTIFS($D$8:$D22,D22,$B$8:$B22,"&lt;&gt;")+1))</f>
+        <f>IF(B22="","",IF($C$5="Snowball",SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22&lt;C22))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($C$8:$C$22=C22)*(ROW($B$8:$B$22)&lt;22))+1,SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22&gt;D22))+SUMPRODUCT(($B$8:$B$22&lt;&gt;"")*($D$8:$D$22=D22)*(ROW($B$8:$B$22)&lt;22))+1))</f>
         <v/>
       </c>
       <c r="G22" s="46">

</xml_diff>